<commit_message>
#5 J6 and J7 Marked DNP Client and JLCPCB.
</commit_message>
<xml_diff>
--- a/Design-Files/NMEA2K-Converter-v1.0/Deliverables/BOM/Client-BOM-v1.0.xlsx
+++ b/Design-Files/NMEA2K-Converter-v1.0/Deliverables/BOM/Client-BOM-v1.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="296">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="297">
   <si>
     <t>#</t>
   </si>
@@ -907,13 +907,16 @@
   </si>
   <si>
     <t>Mosfet</t>
+  </si>
+  <si>
+    <t>DO NOT PLACE</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -952,6 +955,23 @@
     <font>
       <b/>
       <sz val="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="9"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <strike/>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1072,7 +1092,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1111,6 +1131,15 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2205,28 +2234,30 @@
       <c r="C26" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="D26" s="9" t="s">
+      <c r="D26" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="E26" s="10" t="s">
+      <c r="E26" s="16" t="s">
         <v>108</v>
       </c>
-      <c r="F26" s="9" t="s">
+      <c r="F26" s="15" t="s">
         <v>165</v>
       </c>
-      <c r="G26" s="10" t="s">
+      <c r="G26" s="16" t="s">
         <v>203</v>
       </c>
-      <c r="H26" s="9" t="s">
+      <c r="H26" s="15" t="s">
         <v>253</v>
       </c>
-      <c r="I26" s="10" t="s">
+      <c r="I26" s="16" t="s">
         <v>291</v>
       </c>
-      <c r="J26" s="9">
+      <c r="J26" s="15">
         <v>2</v>
       </c>
-      <c r="K26" s="9"/>
+      <c r="K26" s="17" t="s">
+        <v>296</v>
+      </c>
     </row>
     <row r="27" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
@@ -3101,28 +3132,30 @@
       <c r="C54" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="D54" s="9" t="s">
+      <c r="D54" s="15" t="s">
         <v>73</v>
       </c>
-      <c r="E54" s="10" t="s">
+      <c r="E54" s="16" t="s">
         <v>136</v>
       </c>
-      <c r="F54" s="9" t="s">
+      <c r="F54" s="15" t="s">
         <v>173</v>
       </c>
-      <c r="G54" s="10" t="s">
+      <c r="G54" s="16" t="s">
         <v>173</v>
       </c>
-      <c r="H54" s="9" t="s">
+      <c r="H54" s="15" t="s">
         <v>291</v>
       </c>
-      <c r="I54" s="10" t="s">
+      <c r="I54" s="16" t="s">
         <v>291</v>
       </c>
-      <c r="J54" s="9">
+      <c r="J54" s="15">
         <v>1</v>
       </c>
-      <c r="K54" s="9"/>
+      <c r="K54" s="17" t="s">
+        <v>296</v>
+      </c>
     </row>
     <row r="55" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="1"/>

</xml_diff>